<commit_message>
Penambahan login if else dan switch case
</commit_message>
<xml_diff>
--- a/Data Files/Raw Data/login_data.xlsx
+++ b/Data Files/Raw Data/login_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malik\Katalon Studio\Web Automation - Project practice\Data Files\Raw Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malik\git\Exercise-Tema-3-dan-4\Data Files\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9E823C-7EA0-4643-BA47-F53D1120F406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9567414-E003-4CD8-BBA3-B00B3D553DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
-  <si>
-    <t>Password</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>user.test02@gmail.com</t>
   </si>
@@ -40,7 +37,100 @@
     <t>#Secret@404</t>
   </si>
   <si>
-    <t>Username</t>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>qty</t>
+  </si>
+  <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>lastname</t>
+  </si>
+  <si>
+    <t>company</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>postcode</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>test02</t>
+  </si>
+  <si>
+    <t>test03</t>
+  </si>
+  <si>
+    <t>test04</t>
+  </si>
+  <si>
+    <t>test05</t>
+  </si>
+  <si>
+    <t>Bogor</t>
+  </si>
+  <si>
+    <t>Jakarta</t>
+  </si>
+  <si>
+    <t>Bekasi</t>
+  </si>
+  <si>
+    <t>Tanggerang</t>
+  </si>
+  <si>
+    <t>Cibinong</t>
+  </si>
+  <si>
+    <t>Cikini</t>
+  </si>
+  <si>
+    <t>Mustika Jaya</t>
+  </si>
+  <si>
+    <t>Bintaro</t>
+  </si>
+  <si>
+    <t>PT.test02</t>
+  </si>
+  <si>
+    <t>PT.test03</t>
+  </si>
+  <si>
+    <t>PT.test04</t>
+  </si>
+  <si>
+    <t>PT.test05</t>
+  </si>
+  <si>
+    <t>payments</t>
+  </si>
+  <si>
+    <t>Direct Bank Transfer</t>
+  </si>
+  <si>
+    <t>Check Payments</t>
+  </si>
+  <si>
+    <t>Cash on Delivery</t>
   </si>
 </sst>
 </file>
@@ -91,9 +181,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -397,67 +490,227 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="2"/>
+    <col min="12" max="12" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <v>81357296841</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="2">
+        <v>187465</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>85749217306</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="2">
+        <v>187466</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="2">
+        <v>82261589437</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="2">
+        <v>187467</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="2">
+        <v>87833492056</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="2">
+        <v>187468</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{5BA842AF-6587-42B1-9B5E-D630EC76B74F}"/>
-    <hyperlink ref="A3:A6" r:id="rId2" display="user.test02@gmail.com" xr:uid="{F376894D-000A-4A77-B090-6D8B5D8C10FC}"/>
+    <hyperlink ref="A3:A5" r:id="rId2" display="user.test02@gmail.com" xr:uid="{F376894D-000A-4A77-B090-6D8B5D8C10FC}"/>
     <hyperlink ref="A3" r:id="rId3" xr:uid="{C4F2C342-CDB7-42BC-9CED-97D0369B6325}"/>
     <hyperlink ref="A4" r:id="rId4" xr:uid="{467F2E13-5A5D-4365-A2C0-801876419123}"/>
-    <hyperlink ref="A5" r:id="rId5" xr:uid="{738B20AB-DA97-4534-8E60-56FE83C638F3}"/>
-    <hyperlink ref="B2" r:id="rId6" xr:uid="{DABE87AC-5BA1-4B36-8EC4-9CF090F63A4C}"/>
-    <hyperlink ref="B3:B6" r:id="rId7" display="#Secret@404" xr:uid="{201B323A-8461-4DB0-BF75-6D70C9E93463}"/>
+    <hyperlink ref="B2" r:id="rId5" xr:uid="{DABE87AC-5BA1-4B36-8EC4-9CF090F63A4C}"/>
+    <hyperlink ref="B3:B5" r:id="rId6" display="#Secret@404" xr:uid="{201B323A-8461-4DB0-BF75-6D70C9E93463}"/>
+    <hyperlink ref="G2" r:id="rId7" xr:uid="{2E0268AF-04B5-4D39-AD4B-99F5C8AD8B8A}"/>
+    <hyperlink ref="G3:G5" r:id="rId8" display="user.test02@gmail.com" xr:uid="{9A997D80-C634-4169-A81D-A56652441D60}"/>
+    <hyperlink ref="G3" r:id="rId9" xr:uid="{80F58100-AF24-4161-B75C-049C21E4E053}"/>
+    <hyperlink ref="G4" r:id="rId10" xr:uid="{9F61DBC6-6EBC-4A58-93A1-ADCB0027C327}"/>
+    <hyperlink ref="G5" r:id="rId11" xr:uid="{233B7ADE-61B1-40C5-89AD-A0A234EF49DB}"/>
+    <hyperlink ref="A5" r:id="rId12" xr:uid="{738B20AB-DA97-4534-8E60-56FE83C638F3}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>